<commit_message>
feat: tích hợp API nhập chi phí tuyển dụng, cập nhật báo cáo và xuất file Excel đúng bộ lọc
</commit_message>
<xml_diff>
--- a/Bao_cao_thoi_gian_chi_phi_tuyen_dung_20261018.xlsx
+++ b/Bao_cao_thoi_gian_chi_phi_tuyen_dung_20261018.xlsx
@@ -416,7 +416,7 @@
         <v>Ngày xuất báo cáo:</v>
       </c>
       <c r="B3" t="str">
-        <v>14:36:51 18/10/2026</v>
+        <v>15:42:39 18/10/2026</v>
       </c>
     </row>
     <row r="4">
@@ -424,7 +424,7 @@
         <v>Kỳ báo cáo:</v>
       </c>
       <c r="B4" t="str">
-        <v>Toàn kỳ</v>
+        <v>2026-01-01 đến 2026-12-31 (THIS_YEAR)</v>
       </c>
     </row>
     <row r="5">
@@ -432,7 +432,7 @@
         <v>Phòng ban:</v>
       </c>
       <c r="B5" t="str">
-        <v>Tất cả</v>
+        <v>dept-tech</v>
       </c>
     </row>
     <row r="6">
@@ -647,7 +647,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -729,121 +729,16 @@
         <v>Hiệu quả cao</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5">
-        <v>2</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Phòng Phát triển Sản phẩm &amp; Thiết kế</v>
-      </c>
-      <c r="C5">
-        <v>6</v>
-      </c>
-      <c r="D5">
-        <v>6</v>
-      </c>
-      <c r="E5" t="str">
-        <v>100%</v>
-      </c>
-      <c r="F5">
-        <v>26.2</v>
-      </c>
-      <c r="G5">
-        <v>24000000</v>
-      </c>
-      <c r="H5">
-        <v>30000000</v>
-      </c>
-      <c r="I5">
-        <v>54000000</v>
-      </c>
-      <c r="J5">
-        <v>9000000</v>
-      </c>
-      <c r="K5" t="str">
-        <v>Hiệu quả cao</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6">
-        <v>3</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Khối Kinh doanh &amp; Marketing</v>
-      </c>
-      <c r="C6">
-        <v>7</v>
-      </c>
-      <c r="D6">
-        <v>8</v>
-      </c>
-      <c r="E6" t="str">
-        <v>88%</v>
-      </c>
-      <c r="F6">
-        <v>21.5</v>
-      </c>
-      <c r="G6">
-        <v>20400000</v>
-      </c>
-      <c r="H6">
-        <v>21000000</v>
-      </c>
-      <c r="I6">
-        <v>41400000</v>
-      </c>
-      <c r="J6">
-        <v>5914286</v>
-      </c>
-      <c r="K6" t="str">
-        <v>Hiệu quả cao</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7">
-        <v>4</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Khối Vận hành &amp; Nhân sự</v>
-      </c>
-      <c r="C7">
-        <v>3</v>
-      </c>
-      <c r="D7">
-        <v>4</v>
-      </c>
-      <c r="E7" t="str">
-        <v>75%</v>
-      </c>
-      <c r="F7">
-        <v>24</v>
-      </c>
-      <c r="G7">
-        <v>10000000</v>
-      </c>
-      <c r="H7">
-        <v>7400000</v>
-      </c>
-      <c r="I7">
-        <v>17400000</v>
-      </c>
-      <c r="J7">
-        <v>5800000</v>
-      </c>
-      <c r="K7" t="str">
-        <v>Trung bình</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -919,233 +814,9 @@
         <v>CHUYÊN GIA CAO CẤP</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5">
-        <v>2</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Backend Golang Developer</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Khối Công nghệ &amp; Phần mềm</v>
-      </c>
-      <c r="D5">
-        <v>6</v>
-      </c>
-      <c r="E5">
-        <v>36.5</v>
-      </c>
-      <c r="F5">
-        <v>28000000</v>
-      </c>
-      <c r="G5">
-        <v>36000000</v>
-      </c>
-      <c r="H5">
-        <v>64000000</v>
-      </c>
-      <c r="I5">
-        <v>10666667</v>
-      </c>
-      <c r="J5" t="str">
-        <v>CHUYÊN GIA CAO CẤP</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6">
-        <v>3</v>
-      </c>
-      <c r="B6" t="str">
-        <v>DevOps / Cloud Engineer</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Khối Công nghệ &amp; Phần mềm</v>
-      </c>
-      <c r="D6">
-        <v>3</v>
-      </c>
-      <c r="E6">
-        <v>31</v>
-      </c>
-      <c r="F6">
-        <v>12000000</v>
-      </c>
-      <c r="G6">
-        <v>15000000</v>
-      </c>
-      <c r="H6">
-        <v>27000000</v>
-      </c>
-      <c r="I6">
-        <v>9000000</v>
-      </c>
-      <c r="J6" t="str">
-        <v>CHUYÊN GIA CAO CẤP</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7">
-        <v>4</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Product Manager (B2B SaaS)</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Phòng Phát triển Sản phẩm &amp; Thiết kế</v>
-      </c>
-      <c r="D7">
-        <v>2</v>
-      </c>
-      <c r="E7">
-        <v>29.5</v>
-      </c>
-      <c r="F7">
-        <v>10000000</v>
-      </c>
-      <c r="G7">
-        <v>12000000</v>
-      </c>
-      <c r="H7">
-        <v>22000000</v>
-      </c>
-      <c r="I7">
-        <v>11000000</v>
-      </c>
-      <c r="J7" t="str">
-        <v>CHUYÊN GIA CAO CẤP</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8">
-        <v>5</v>
-      </c>
-      <c r="B8" t="str">
-        <v>UI/UX Product Designer</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Phòng Phát triển Sản phẩm &amp; Thiết kế</v>
-      </c>
-      <c r="D8">
-        <v>4</v>
-      </c>
-      <c r="E8">
-        <v>24.5</v>
-      </c>
-      <c r="F8">
-        <v>14000000</v>
-      </c>
-      <c r="G8">
-        <v>18000000</v>
-      </c>
-      <c r="H8">
-        <v>32000000</v>
-      </c>
-      <c r="I8">
-        <v>8000000</v>
-      </c>
-      <c r="J8" t="str">
-        <v>TRUNG BÌNH</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>6</v>
-      </c>
-      <c r="B9" t="str">
-        <v>B2B Sales Enterprise Lead</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Khối Kinh doanh &amp; Marketing</v>
-      </c>
-      <c r="D9">
-        <v>4</v>
-      </c>
-      <c r="E9">
-        <v>22</v>
-      </c>
-      <c r="F9">
-        <v>11400000</v>
-      </c>
-      <c r="G9">
-        <v>12000000</v>
-      </c>
-      <c r="H9">
-        <v>23400000</v>
-      </c>
-      <c r="I9">
-        <v>5850000</v>
-      </c>
-      <c r="J9" t="str">
-        <v>TRUNG BÌNH</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>7</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Digital Marketing Specialist</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Khối Kinh doanh &amp; Marketing</v>
-      </c>
-      <c r="D10">
-        <v>3</v>
-      </c>
-      <c r="E10">
-        <v>20.8</v>
-      </c>
-      <c r="F10">
-        <v>9000000</v>
-      </c>
-      <c r="G10">
-        <v>9000000</v>
-      </c>
-      <c r="H10">
-        <v>18000000</v>
-      </c>
-      <c r="I10">
-        <v>6000000</v>
-      </c>
-      <c r="J10" t="str">
-        <v>TIÊU CHUẨN</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <v>8</v>
-      </c>
-      <c r="B11" t="str">
-        <v>HR Operations &amp; Talent Specialist</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Khối Vận hành &amp; Nhân sự</v>
-      </c>
-      <c r="D11">
-        <v>3</v>
-      </c>
-      <c r="E11">
-        <v>24</v>
-      </c>
-      <c r="F11">
-        <v>10000000</v>
-      </c>
-      <c r="G11">
-        <v>7400000</v>
-      </c>
-      <c r="H11">
-        <v>17400000</v>
-      </c>
-      <c r="I11">
-        <v>5800000</v>
-      </c>
-      <c r="J11" t="str">
-        <v>TIÊU CHUẨN</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>